<commit_message>
Updated wind, solar, and electrolyzer costs
</commit_message>
<xml_diff>
--- a/src/ereznic2/H2_Analysis/green_steel_site_renewable_costs_ATB_aug2024.xlsx
+++ b/src/ereznic2/H2_Analysis/green_steel_site_renewable_costs_ATB_aug2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ereznic2\Documents\GreenSteel\src\ereznic2\H2_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8E16F2-53EF-430E-ACB6-2097C8796D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB088EEE-04E0-47DF-81C4-D2672CEAFD85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3456" yWindow="2772" windowWidth="15396" windowHeight="14508" xr2:uid="{6F370ACC-2FEA-4034-9DAD-6260C657696D}"/>
+    <workbookView xWindow="20544" yWindow="0" windowWidth="20832" windowHeight="17376" xr2:uid="{6F370ACC-2FEA-4034-9DAD-6260C657696D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -821,19 +821,19 @@
         <v>49</v>
       </c>
       <c r="B9" s="4">
-        <v>1666</v>
+        <v>1472</v>
       </c>
       <c r="C9" s="4">
-        <v>1666</v>
+        <v>1472</v>
       </c>
       <c r="D9" s="6">
-        <v>1803</v>
+        <v>1601</v>
       </c>
       <c r="E9" s="4">
-        <v>2335</v>
+        <v>2103</v>
       </c>
       <c r="F9" s="4">
-        <v>1666</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -841,19 +841,19 @@
         <v>20</v>
       </c>
       <c r="B10" s="4">
-        <v>1569</v>
+        <v>1380</v>
       </c>
       <c r="C10" s="4">
-        <v>1569</v>
+        <v>1380</v>
       </c>
       <c r="D10" s="6">
-        <v>1703</v>
+        <v>1507</v>
       </c>
       <c r="E10" s="4">
-        <v>2151</v>
+        <v>1929</v>
       </c>
       <c r="F10" s="4">
-        <v>1569</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -861,19 +861,19 @@
         <v>21</v>
       </c>
       <c r="B11" s="4">
-        <v>1408</v>
+        <v>1228</v>
       </c>
       <c r="C11" s="4">
-        <v>1408</v>
+        <v>1228</v>
       </c>
       <c r="D11" s="1">
-        <v>1537</v>
+        <v>1350</v>
       </c>
       <c r="E11" s="4">
-        <v>1844</v>
+        <v>1640</v>
       </c>
       <c r="F11" s="4">
-        <v>1408</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -881,19 +881,19 @@
         <v>22</v>
       </c>
       <c r="B12" s="4">
-        <v>1335</v>
+        <v>1159</v>
       </c>
       <c r="C12" s="4">
-        <v>1335</v>
+        <v>1159</v>
       </c>
       <c r="D12" s="1">
-        <v>1457</v>
+        <v>1275</v>
       </c>
       <c r="E12" s="4">
-        <v>1749</v>
+        <v>1550</v>
       </c>
       <c r="F12" s="4">
-        <v>1335</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -901,19 +901,19 @@
         <v>23</v>
       </c>
       <c r="B13" s="4">
-        <v>1115</v>
+        <v>952</v>
       </c>
       <c r="C13" s="4">
-        <v>1115</v>
+        <v>952</v>
       </c>
       <c r="D13" s="1">
-        <v>1219</v>
+        <v>1050</v>
       </c>
       <c r="E13" s="4">
-        <v>1463</v>
+        <v>1281</v>
       </c>
       <c r="F13" s="4">
-        <v>1115</v>
+        <v>952</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -1069,19 +1069,19 @@
         <v>51</v>
       </c>
       <c r="B22" s="4">
-        <v>1483</v>
+        <v>1367</v>
       </c>
       <c r="C22" s="4">
-        <v>1483</v>
+        <v>1367</v>
       </c>
       <c r="D22" s="4">
-        <v>1483</v>
+        <v>1367</v>
       </c>
       <c r="E22" s="4">
-        <v>1483</v>
+        <v>1367</v>
       </c>
       <c r="F22" s="4">
-        <v>1483</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -1089,19 +1089,19 @@
         <v>30</v>
       </c>
       <c r="B23" s="4">
-        <v>1492</v>
+        <v>1323</v>
       </c>
       <c r="C23" s="4">
-        <v>1492</v>
+        <v>1323</v>
       </c>
       <c r="D23" s="4">
-        <v>1492</v>
+        <v>1323</v>
       </c>
       <c r="E23" s="4">
-        <v>1492</v>
+        <v>1323</v>
       </c>
       <c r="F23" s="4">
-        <v>1492</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -1109,19 +1109,19 @@
         <v>31</v>
       </c>
       <c r="B24" s="4">
-        <v>1193</v>
+        <v>1044</v>
       </c>
       <c r="C24" s="4">
-        <v>1193</v>
+        <v>1044</v>
       </c>
       <c r="D24" s="4">
-        <v>1193</v>
+        <v>1044</v>
       </c>
       <c r="E24" s="4">
-        <v>1193</v>
+        <v>1044</v>
       </c>
       <c r="F24" s="4">
-        <v>1193</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1129,19 +1129,19 @@
         <v>32</v>
       </c>
       <c r="B25" s="4">
-        <v>895</v>
+        <v>764</v>
       </c>
       <c r="C25" s="4">
-        <v>895</v>
+        <v>764</v>
       </c>
       <c r="D25" s="4">
-        <v>895</v>
+        <v>764</v>
       </c>
       <c r="E25" s="4">
-        <v>895</v>
+        <v>764</v>
       </c>
       <c r="F25" s="4">
-        <v>895</v>
+        <v>764</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -1149,19 +1149,19 @@
         <v>33</v>
       </c>
       <c r="B26" s="4">
-        <v>683</v>
+        <v>559</v>
       </c>
       <c r="C26" s="4">
-        <v>683</v>
+        <v>559</v>
       </c>
       <c r="D26" s="4">
-        <v>683</v>
+        <v>559</v>
       </c>
       <c r="E26" s="4">
-        <v>683</v>
+        <v>559</v>
       </c>
       <c r="F26" s="4">
-        <v>683</v>
+        <v>559</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -1453,4 +1453,10 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>